<commit_message>
fix: add Athgaon and Bistupur to CakeZone mapping
These two locations were missing from the mapping but present in the
data. Added both to the East zone as requested by user.
</commit_message>
<xml_diff>
--- a/cakezone_zone_city_mapping.xlsx
+++ b/cakezone_zone_city_mapping.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="253">
   <si>
     <t>Store Name</t>
   </si>
@@ -580,6 +580,12 @@
     <t>Colaba - Cake Zone - Online</t>
   </si>
   <si>
+    <t>Athgaon - Cake Zone - Online</t>
+  </si>
+  <si>
+    <t>Bistupur - Cake Zone - Online</t>
+  </si>
+  <si>
     <t>Ludhiana</t>
   </si>
   <si>
@@ -749,6 +755,12 @@
   </si>
   <si>
     <t>Patna</t>
+  </si>
+  <si>
+    <t>Guwahati</t>
+  </si>
+  <si>
+    <t>Jamshedpur</t>
   </si>
   <si>
     <t>North</t>
@@ -1092,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C186"/>
+  <dimension ref="A1:C188"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1111,10 +1123,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1122,10 +1134,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1133,10 +1145,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1144,10 +1156,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1155,10 +1167,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C6" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1166,10 +1178,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C7" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1177,10 +1189,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C8" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1188,10 +1200,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1199,10 +1211,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C10" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1210,10 +1222,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C11" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1221,10 +1233,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C12" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1232,10 +1244,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C13" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1243,10 +1255,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C14" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1254,10 +1266,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C15" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1265,10 +1277,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C16" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1276,10 +1288,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C17" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1287,10 +1299,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C18" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1298,10 +1310,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C19" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1309,10 +1321,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C20" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1320,10 +1332,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C21" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1331,10 +1343,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C22" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1342,10 +1354,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C23" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1353,10 +1365,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C24" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1364,10 +1376,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C25" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1375,10 +1387,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C26" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1386,10 +1398,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1397,10 +1409,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C28" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1408,10 +1420,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C29" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1419,10 +1431,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C30" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1430,10 +1442,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C31" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1441,10 +1453,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C32" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1452,10 +1464,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C33" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1463,10 +1475,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C34" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1474,10 +1486,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C35" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1485,10 +1497,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C36" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1496,10 +1508,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C37" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1507,10 +1519,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C38" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1518,10 +1530,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C39" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1529,10 +1541,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C40" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1540,10 +1552,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C41" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1551,10 +1563,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C42" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1562,10 +1574,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C43" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1573,10 +1585,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C44" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1584,10 +1596,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C45" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1595,10 +1607,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C46" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1606,10 +1618,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C47" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1617,10 +1629,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C48" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1628,10 +1640,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C49" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1639,10 +1651,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C50" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1650,10 +1662,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C51" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1661,10 +1673,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C52" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1672,10 +1684,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C53" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1683,10 +1695,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C54" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1694,10 +1706,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C55" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1705,10 +1717,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C56" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1716,10 +1728,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C57" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1727,10 +1739,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C58" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1738,10 +1750,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C59" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1749,10 +1761,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C60" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1760,10 +1772,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C61" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1771,10 +1783,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C62" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1782,10 +1794,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C63" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1793,10 +1805,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C64" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1804,10 +1816,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C65" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1815,10 +1827,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C66" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1826,10 +1838,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C67" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1837,10 +1849,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C68" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1848,10 +1860,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C69" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1859,10 +1871,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C70" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1870,10 +1882,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C71" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1881,10 +1893,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C72" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1892,10 +1904,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C73" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1903,10 +1915,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C74" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1914,10 +1926,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C75" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1925,10 +1937,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C76" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1936,10 +1948,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C77" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1947,10 +1959,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C78" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1958,10 +1970,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C79" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1969,10 +1981,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C80" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -1980,10 +1992,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C81" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -1991,10 +2003,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C82" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2002,10 +2014,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C83" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2013,10 +2025,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C84" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2024,10 +2036,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C85" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2035,10 +2047,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C86" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2046,10 +2058,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C87" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2057,10 +2069,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C88" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2068,10 +2080,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C89" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2079,10 +2091,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C90" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2090,10 +2102,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C91" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2101,10 +2113,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C92" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2112,10 +2124,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C93" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2123,10 +2135,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C94" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2134,10 +2146,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C95" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2145,10 +2157,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C96" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2156,10 +2168,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C97" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2167,10 +2179,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C98" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2178,10 +2190,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C99" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2189,10 +2201,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C100" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2200,10 +2212,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C101" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2211,10 +2223,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C102" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2222,10 +2234,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C103" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2233,10 +2245,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C104" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2244,10 +2256,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C105" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2255,10 +2267,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C106" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2266,10 +2278,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C107" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2277,10 +2289,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C108" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2288,10 +2300,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C109" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2299,10 +2311,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C110" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2310,10 +2322,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C111" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2321,10 +2333,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C112" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2332,10 +2344,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C113" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2343,10 +2355,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C114" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2354,10 +2366,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C115" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2365,10 +2377,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C116" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2376,10 +2388,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C117" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2387,10 +2399,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C118" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2398,10 +2410,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C119" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2409,10 +2421,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C120" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2420,10 +2432,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C121" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2431,10 +2443,10 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C122" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2442,10 +2454,10 @@
         <v>124</v>
       </c>
       <c r="B123" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C123" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2453,10 +2465,10 @@
         <v>125</v>
       </c>
       <c r="B124" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C124" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2464,10 +2476,10 @@
         <v>126</v>
       </c>
       <c r="B125" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C125" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2475,10 +2487,10 @@
         <v>127</v>
       </c>
       <c r="B126" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C126" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -2486,10 +2498,10 @@
         <v>128</v>
       </c>
       <c r="B127" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C127" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -2497,10 +2509,10 @@
         <v>129</v>
       </c>
       <c r="B128" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C128" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -2508,10 +2520,10 @@
         <v>130</v>
       </c>
       <c r="B129" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C129" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -2519,10 +2531,10 @@
         <v>131</v>
       </c>
       <c r="B130" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C130" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -2530,10 +2542,10 @@
         <v>132</v>
       </c>
       <c r="B131" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C131" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -2541,10 +2553,10 @@
         <v>133</v>
       </c>
       <c r="B132" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C132" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -2552,10 +2564,10 @@
         <v>134</v>
       </c>
       <c r="B133" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C133" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -2563,10 +2575,10 @@
         <v>135</v>
       </c>
       <c r="B134" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C134" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -2574,10 +2586,10 @@
         <v>136</v>
       </c>
       <c r="B135" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C135" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -2585,10 +2597,10 @@
         <v>137</v>
       </c>
       <c r="B136" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C136" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -2596,10 +2608,10 @@
         <v>138</v>
       </c>
       <c r="B137" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C137" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -2607,10 +2619,10 @@
         <v>139</v>
       </c>
       <c r="B138" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C138" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -2618,10 +2630,10 @@
         <v>140</v>
       </c>
       <c r="B139" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C139" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="140" spans="1:3">
@@ -2629,10 +2641,10 @@
         <v>141</v>
       </c>
       <c r="B140" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C140" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -2640,10 +2652,10 @@
         <v>142</v>
       </c>
       <c r="B141" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C141" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="142" spans="1:3">
@@ -2651,10 +2663,10 @@
         <v>143</v>
       </c>
       <c r="B142" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C142" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -2662,10 +2674,10 @@
         <v>144</v>
       </c>
       <c r="B143" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C143" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -2673,10 +2685,10 @@
         <v>145</v>
       </c>
       <c r="B144" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C144" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -2684,10 +2696,10 @@
         <v>146</v>
       </c>
       <c r="B145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C145" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -2695,10 +2707,10 @@
         <v>147</v>
       </c>
       <c r="B146" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C146" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -2706,10 +2718,10 @@
         <v>148</v>
       </c>
       <c r="B147" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C147" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="148" spans="1:3">
@@ -2717,10 +2729,10 @@
         <v>149</v>
       </c>
       <c r="B148" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C148" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="149" spans="1:3">
@@ -2728,10 +2740,10 @@
         <v>150</v>
       </c>
       <c r="B149" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C149" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="150" spans="1:3">
@@ -2739,10 +2751,10 @@
         <v>151</v>
       </c>
       <c r="B150" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C150" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -2750,10 +2762,10 @@
         <v>152</v>
       </c>
       <c r="B151" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C151" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -2761,10 +2773,10 @@
         <v>153</v>
       </c>
       <c r="B152" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C152" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -2772,10 +2784,10 @@
         <v>154</v>
       </c>
       <c r="B153" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C153" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -2783,10 +2795,10 @@
         <v>155</v>
       </c>
       <c r="B154" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C154" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="155" spans="1:3">
@@ -2794,10 +2806,10 @@
         <v>156</v>
       </c>
       <c r="B155" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C155" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -2805,10 +2817,10 @@
         <v>157</v>
       </c>
       <c r="B156" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C156" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="157" spans="1:3">
@@ -2816,10 +2828,10 @@
         <v>158</v>
       </c>
       <c r="B157" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C157" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -2827,10 +2839,10 @@
         <v>159</v>
       </c>
       <c r="B158" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C158" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -2838,10 +2850,10 @@
         <v>160</v>
       </c>
       <c r="B159" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C159" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="160" spans="1:3">
@@ -2849,10 +2861,10 @@
         <v>161</v>
       </c>
       <c r="B160" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C160" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -2860,10 +2872,10 @@
         <v>162</v>
       </c>
       <c r="B161" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C161" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="162" spans="1:3">
@@ -2871,10 +2883,10 @@
         <v>163</v>
       </c>
       <c r="B162" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C162" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -2882,10 +2894,10 @@
         <v>164</v>
       </c>
       <c r="B163" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C163" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -2893,10 +2905,10 @@
         <v>165</v>
       </c>
       <c r="B164" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C164" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -2904,10 +2916,10 @@
         <v>166</v>
       </c>
       <c r="B165" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C165" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="166" spans="1:3">
@@ -2915,10 +2927,10 @@
         <v>167</v>
       </c>
       <c r="B166" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C166" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -2926,10 +2938,10 @@
         <v>168</v>
       </c>
       <c r="B167" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C167" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="168" spans="1:3">
@@ -2937,10 +2949,10 @@
         <v>169</v>
       </c>
       <c r="B168" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C168" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="169" spans="1:3">
@@ -2948,10 +2960,10 @@
         <v>170</v>
       </c>
       <c r="B169" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C169" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -2959,10 +2971,10 @@
         <v>171</v>
       </c>
       <c r="B170" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C170" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -2970,10 +2982,10 @@
         <v>172</v>
       </c>
       <c r="B171" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C171" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -2981,10 +2993,10 @@
         <v>173</v>
       </c>
       <c r="B172" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C172" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -2992,10 +3004,10 @@
         <v>174</v>
       </c>
       <c r="B173" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C173" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="174" spans="1:3">
@@ -3003,10 +3015,10 @@
         <v>175</v>
       </c>
       <c r="B174" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C174" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -3014,10 +3026,10 @@
         <v>176</v>
       </c>
       <c r="B175" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C175" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -3025,10 +3037,10 @@
         <v>177</v>
       </c>
       <c r="B176" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C176" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -3036,10 +3048,10 @@
         <v>178</v>
       </c>
       <c r="B177" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C177" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -3047,10 +3059,10 @@
         <v>179</v>
       </c>
       <c r="B178" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C178" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -3058,10 +3070,10 @@
         <v>180</v>
       </c>
       <c r="B179" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C179" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -3069,10 +3081,10 @@
         <v>181</v>
       </c>
       <c r="B180" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C180" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -3080,10 +3092,10 @@
         <v>182</v>
       </c>
       <c r="B181" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C181" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -3091,10 +3103,10 @@
         <v>183</v>
       </c>
       <c r="B182" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C182" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -3102,10 +3114,10 @@
         <v>184</v>
       </c>
       <c r="B183" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C183" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -3113,10 +3125,10 @@
         <v>185</v>
       </c>
       <c r="B184" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C184" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -3124,10 +3136,10 @@
         <v>186</v>
       </c>
       <c r="B185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C185" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -3135,10 +3147,32 @@
         <v>187</v>
       </c>
       <c r="B186" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C186" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3">
+      <c r="A187" t="s">
+        <v>188</v>
+      </c>
+      <c r="B187" t="s">
         <v>247</v>
+      </c>
+      <c r="C187" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
+      <c r="A188" t="s">
+        <v>189</v>
+      </c>
+      <c r="B188" t="s">
+        <v>248</v>
+      </c>
+      <c r="C188" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>